<commit_message>
Update project and tests
</commit_message>
<xml_diff>
--- a/frontend/static/templates/PM_GSS_Side_Template.xlsx
+++ b/frontend/static/templates/PM_GSS_Side_Template.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Optional. How many units the plant has. Blank = the plant's Unit configuration or Equipment Register. ACCB Panel (ACCB-1 + ACCB-2) and Miscellaneous are always one job per plant.</t>
+          <t>Optional. How many units the plant has. Blank = the plant's Unit configuration or Equipment Register. ACCB Panel (ACCB-1 + ACCB-2), Aux. Transformer, ACDB and Miscellaneous are always one job per plant.</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Optional. Added to the log of every task the row creates.</t>
+          <t>Optional. Added to the log of every task the row creates. For Miscellaneous, list the items the job covers (pre-filled: Street Light, ERT — remove or add items).</t>
         </is>
       </c>
     </row>

</xml_diff>